<commit_message>
Cap nhat code extract va file test moi
</commit_message>
<xml_diff>
--- a/code/extracted_data_final.xlsx
+++ b/code/extracted_data_final.xlsx
@@ -464,20 +464,20 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026_07_10_13_00_49_11_case01_T0_P0.png</t>
+          <t>2026_07_09_10_11_36_11_case01_T0_P0.png</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>58.507</v>
+        <v>57.829</v>
       </c>
       <c r="D2" t="n">
-        <v>15.57</v>
+        <v>16.6</v>
       </c>
       <c r="E2" t="n">
-        <v>1.115</v>
+        <v>1.168</v>
       </c>
       <c r="F2" t="n">
-        <v>1.258</v>
+        <v>1.353</v>
       </c>
     </row>
     <row r="3">
@@ -486,20 +486,20 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026_07_10_13_16_28_11_case01_T0_P0.png</t>
+          <t>2026_07_09_10_26_33_11_case01_T0_P0.png</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>58.4315</v>
+        <v>232.772</v>
       </c>
       <c r="D3" t="n">
-        <v>1</v>
+        <v>14.61</v>
       </c>
       <c r="E3" t="n">
-        <v>1.115</v>
+        <v>1.205</v>
       </c>
       <c r="F3" t="n">
-        <v>1.259</v>
+        <v>1.405</v>
       </c>
     </row>
     <row r="4">
@@ -508,18 +508,20 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026_07_10_13_31_25_11_case01_T0_P0.png</t>
+          <t>2026_07_09_10_42_39_11_case01_T0_P0.png</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>58.404</v>
+        <v>58.463</v>
       </c>
       <c r="D4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E4" t="inlineStr"/>
+        <v>16.13</v>
+      </c>
+      <c r="E4" t="n">
+        <v>1.211</v>
+      </c>
       <c r="F4" t="n">
-        <v>1.253</v>
+        <v>1.41</v>
       </c>
     </row>
     <row r="5">
@@ -528,18 +530,20 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026_07_10_13_45_50_11_case01_T0_P0.png</t>
+          <t>2026_07_09_11_37_44_11_case01_T0_P0.png</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>58.583</v>
+        <v>57.828</v>
       </c>
       <c r="D5" t="n">
-        <v>14.24</v>
-      </c>
-      <c r="E5" t="inlineStr"/>
+        <v>16.56</v>
+      </c>
+      <c r="E5" t="n">
+        <v>1.2</v>
+      </c>
       <c r="F5" t="n">
-        <v>1.299</v>
+        <v>1.398</v>
       </c>
     </row>
     <row r="6">
@@ -548,18 +552,20 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026_07_10_14_00_53_11_case01_T0_P0.png</t>
+          <t>2026_07_09_12_08_15_11_case01_T0_P0.png</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>59.024</v>
+        <v>58.065</v>
       </c>
       <c r="D6" t="n">
-        <v>1</v>
-      </c>
-      <c r="E6" t="inlineStr"/>
+        <v>16.64</v>
+      </c>
+      <c r="E6" t="n">
+        <v>1.35</v>
+      </c>
       <c r="F6" t="n">
-        <v>1.291</v>
+        <v>1.3915</v>
       </c>
     </row>
   </sheetData>
@@ -614,15 +620,21 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026_07_10_13_11_35_11_case12_T32_P0.png</t>
+          <t>2026_07_09_10_21_18_11_case12_T32_P0.png</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>57.3</v>
-      </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
+        <v>17.431</v>
+      </c>
+      <c r="D2" t="n">
+        <v>16.69</v>
+      </c>
+      <c r="E2" t="n">
+        <v>2.039</v>
+      </c>
+      <c r="F2" t="n">
+        <v>2.55</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -630,13 +642,21 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026_07_10_13_27_13_11_case12_T32_P0.png</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
+          <t>2026_07_09_10_36_15_11_case12_T32_P0.png</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>17.497</v>
+      </c>
+      <c r="D3" t="n">
+        <v>14.73</v>
+      </c>
+      <c r="E3" t="n">
+        <v>2.158</v>
+      </c>
+      <c r="F3" t="n">
+        <v>2.696</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -644,13 +664,21 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026_07_10_13_42_12_11_case12_T32_P0.png</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
+          <t>2026_07_09_10_52_23_11_case12_T32_P0.png</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>17.66</v>
+      </c>
+      <c r="D4" t="n">
+        <v>16.13</v>
+      </c>
+      <c r="E4" t="n">
+        <v>2.133</v>
+      </c>
+      <c r="F4" t="n">
+        <v>2.685</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -658,16 +686,20 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026_07_10_13_56_37_11_case12_T32_P0.png</t>
+          <t>2026_07_09_11_48_26_11_case12_T32_P0.png</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>17.479</v>
-      </c>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
+        <v>17.54</v>
+      </c>
+      <c r="D5" t="n">
+        <v>16.78</v>
+      </c>
+      <c r="E5" t="n">
+        <v>2.252</v>
+      </c>
       <c r="F5" t="n">
-        <v>2.995</v>
+        <v>2.774</v>
       </c>
     </row>
     <row r="6">
@@ -676,13 +708,21 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026_07_10_14_11_39_11_case12_T32_P0.png</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
+          <t>2026_07_09_12_18_56_11_case12_T32_P0.png</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>40.369</v>
+      </c>
+      <c r="D6" t="n">
+        <v>16.82</v>
+      </c>
+      <c r="E6" t="n">
+        <v>2.274</v>
+      </c>
+      <c r="F6" t="n">
+        <v>2.794</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -736,15 +776,21 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026_07_10_13_12_19_11_case13_T40_P0.png</t>
+          <t>2026_07_09_10_22_02_11_case13_T40_P0.png</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>57.31</v>
-      </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
+        <v>40.707</v>
+      </c>
+      <c r="D2" t="n">
+        <v>16.57</v>
+      </c>
+      <c r="E2" t="n">
+        <v>2.036</v>
+      </c>
+      <c r="F2" t="n">
+        <v>2.549</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -752,13 +798,21 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026_07_10_13_27_58_11_case13_T40_P0.png</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
+          <t>2026_07_09_10_37_00_11_case13_T40_P0.png</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>41.799</v>
+      </c>
+      <c r="D3" t="n">
+        <v>14.67</v>
+      </c>
+      <c r="E3" t="n">
+        <v>2.16</v>
+      </c>
+      <c r="F3" t="n">
+        <v>2.698</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -766,15 +820,21 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026_07_10_13_42_56_11_case13_T40_P0.png</t>
+          <t>2026_07_09_10_53_08_11_case13_T40_P0.png</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>5735</v>
-      </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
+        <v>17.626</v>
+      </c>
+      <c r="D4" t="n">
+        <v>16.06</v>
+      </c>
+      <c r="E4" t="n">
+        <v>2.16</v>
+      </c>
+      <c r="F4" t="n">
+        <v>2.703</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -782,13 +842,21 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026_07_10_13_57_22_11_case13_T40_P0.png</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
+          <t>2026_07_09_11_49_11_11_case13_T40_P0.png</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>17.462</v>
+      </c>
+      <c r="D5" t="n">
+        <v>16.77</v>
+      </c>
+      <c r="E5" t="n">
+        <v>2.264</v>
+      </c>
+      <c r="F5" t="n">
+        <v>2.787</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -796,13 +864,21 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026_07_10_14_12_23_11_case13_T40_P0.png</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
+          <t>2026_07_09_12_19_41_11_case13_T40_P0.png</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>17.505</v>
+      </c>
+      <c r="D6" t="n">
+        <v>16.82</v>
+      </c>
+      <c r="E6" t="n">
+        <v>2.288</v>
+      </c>
+      <c r="F6" t="n">
+        <v>2.809</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -856,18 +932,20 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026_07_10_13_02_27_11_case02_T2_P0.png</t>
+          <t>2026_07_09_10_13_15_11_case02_T2_P0.png</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>58.505</v>
+        <v>57.828</v>
       </c>
       <c r="D2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E2" t="inlineStr"/>
+        <v>16.72</v>
+      </c>
+      <c r="E2" t="n">
+        <v>1.184</v>
+      </c>
       <c r="F2" t="n">
-        <v>1.239</v>
+        <v>1.367</v>
       </c>
     </row>
     <row r="3">
@@ -876,18 +954,20 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026_07_10_13_18_07_11_case02_T2_P0.png</t>
+          <t>2026_07_09_10_28_12_11_case02_T2_P0.png</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>58.4195</v>
+        <v>57.675</v>
       </c>
       <c r="D3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E3" t="inlineStr"/>
+        <v>14.7</v>
+      </c>
+      <c r="E3" t="n">
+        <v>1.238</v>
+      </c>
       <c r="F3" t="n">
-        <v>1</v>
+        <v>1.432</v>
       </c>
     </row>
     <row r="4">
@@ -896,18 +976,20 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026_07_10_13_33_04_11_case02_T2_P0.png</t>
+          <t>2026_07_09_10_44_18_11_case02_T2_P0.png</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>58.3955</v>
+        <v>58.462</v>
       </c>
       <c r="D4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E4" t="inlineStr"/>
+        <v>16.18</v>
+      </c>
+      <c r="E4" t="n">
+        <v>1.215</v>
+      </c>
       <c r="F4" t="n">
-        <v>1.273</v>
+        <v>1.413</v>
       </c>
     </row>
     <row r="5">
@@ -916,18 +998,20 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026_07_10_13_47_30_11_case02_T2_P0.png</t>
+          <t>2026_07_09_11_39_23_11_case02_T2_P0.png</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>58.607</v>
+        <v>58.055</v>
       </c>
       <c r="D5" t="n">
-        <v>1</v>
-      </c>
-      <c r="E5" t="inlineStr"/>
+        <v>16.62</v>
+      </c>
+      <c r="E5" t="n">
+        <v>1.199</v>
+      </c>
       <c r="F5" t="n">
-        <v>1.317</v>
+        <v>1.397</v>
       </c>
     </row>
     <row r="6">
@@ -936,18 +1020,20 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026_07_10_14_02_32_11_case02_T2_P0.png</t>
+          <t>2026_07_09_12_09_54_11_case02_T2_P0.png</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>59.037</v>
+        <v>57.828</v>
       </c>
       <c r="D6" t="n">
-        <v>1</v>
-      </c>
-      <c r="E6" t="inlineStr"/>
+        <v>16.75</v>
+      </c>
+      <c r="E6" t="n">
+        <v>1.373</v>
+      </c>
       <c r="F6" t="n">
-        <v>1.268</v>
+        <v>1.548</v>
       </c>
     </row>
   </sheetData>
@@ -1002,18 +1088,20 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026_07_10_13_04_06_11_case03_T4_P1.png</t>
+          <t>2026_07_09_10_14_52_11_case03_T4_P1.png</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>58.3475</v>
+        <v>57.579</v>
       </c>
       <c r="D2" t="n">
-        <v>15.57</v>
-      </c>
-      <c r="E2" t="inlineStr"/>
+        <v>16.63</v>
+      </c>
+      <c r="E2" t="n">
+        <v>1.191</v>
+      </c>
       <c r="F2" t="n">
-        <v>1.195</v>
+        <v>1.371</v>
       </c>
     </row>
     <row r="3">
@@ -1022,16 +1110,20 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026_07_10_13_19_46_11_case03_T4_P1.png</t>
+          <t>2026_07_09_10_29_51_11_case03_T4_P1.png</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>58.2825</v>
-      </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
+        <v>57.92</v>
+      </c>
+      <c r="D3" t="n">
+        <v>14.67</v>
+      </c>
+      <c r="E3" t="n">
+        <v>1.218</v>
+      </c>
       <c r="F3" t="n">
-        <v>1.174</v>
+        <v>1.412</v>
       </c>
     </row>
     <row r="4">
@@ -1040,16 +1132,20 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026_07_10_13_34_42_11_case03_T4_P1.png</t>
+          <t>2026_07_09_10_45_57_11_case03_T4_P1.png</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>58.2685</v>
-      </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
+        <v>58.455</v>
+      </c>
+      <c r="D4" t="n">
+        <v>16.08</v>
+      </c>
+      <c r="E4" t="n">
+        <v>1.211</v>
+      </c>
       <c r="F4" t="n">
-        <v>1.206</v>
+        <v>1.408</v>
       </c>
     </row>
     <row r="5">
@@ -1058,14 +1154,20 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026_07_10_13_49_09_11_case03_T4_P1.png</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
+          <t>2026_07_09_11_41_02_11_case03_T4_P1.png</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>58.035</v>
+      </c>
+      <c r="D5" t="n">
+        <v>16.6</v>
+      </c>
+      <c r="E5" t="n">
+        <v>1.21</v>
+      </c>
       <c r="F5" t="n">
-        <v>1.25</v>
+        <v>1.408</v>
       </c>
     </row>
     <row r="6">
@@ -1074,14 +1176,20 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026_07_10_14_04_11_11_case03_T4_P1.png</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
+          <t>2026_07_09_12_11_33_11_case03_T4_P1.png</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>58.047</v>
+      </c>
+      <c r="D6" t="n">
+        <v>16.71</v>
+      </c>
+      <c r="E6" t="n">
+        <v>1.365</v>
+      </c>
       <c r="F6" t="n">
-        <v>1.212</v>
+        <v>1.545</v>
       </c>
     </row>
   </sheetData>
@@ -1136,18 +1244,20 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026_07_10_13_05_37_11_case04_T6_P0.png</t>
+          <t>2026_07_09_10_16_24_11_case04_T6_P0.png</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>52.0515</v>
+        <v>51.0145</v>
       </c>
       <c r="D2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E2" t="inlineStr"/>
+        <v>16.69</v>
+      </c>
+      <c r="E2" t="n">
+        <v>1.13</v>
+      </c>
       <c r="F2" t="n">
-        <v>1.279</v>
+        <v>1.291</v>
       </c>
     </row>
     <row r="3">
@@ -1156,18 +1266,20 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026_07_10_13_21_17_11_case04_T6_P0.png</t>
+          <t>2026_07_09_10_31_22_11_case04_T6_P0.png</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>51.985</v>
+        <v>51.088</v>
       </c>
       <c r="D3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E3" t="inlineStr"/>
+        <v>14.6</v>
+      </c>
+      <c r="E3" t="n">
+        <v>1.153</v>
+      </c>
       <c r="F3" t="n">
-        <v>1.27</v>
+        <v>1.322</v>
       </c>
     </row>
     <row r="4">
@@ -1176,18 +1288,20 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026_07_10_13_36_14_11_case04_T6_P0.png</t>
+          <t>2026_07_09_10_47_28_11_case04_T6_P0.png</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>51.9675</v>
+        <v>51.782</v>
       </c>
       <c r="D4" t="n">
-        <v>14.95</v>
-      </c>
-      <c r="E4" t="inlineStr"/>
+        <v>16.2</v>
+      </c>
+      <c r="E4" t="n">
+        <v>1.137</v>
+      </c>
       <c r="F4" t="n">
-        <v>1.32</v>
+        <v>1.311</v>
       </c>
     </row>
     <row r="5">
@@ -1196,18 +1310,20 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026_07_10_13_50_40_11_case04_T6_P0.png</t>
+          <t>2026_07_09_11_42_33_11_case04_T6_P0.png</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>52.139</v>
+        <v>51.414</v>
       </c>
       <c r="D5" t="n">
-        <v>1</v>
-      </c>
-      <c r="E5" t="inlineStr"/>
+        <v>16.65</v>
+      </c>
+      <c r="E5" t="n">
+        <v>1.155</v>
+      </c>
       <c r="F5" t="n">
-        <v>1.345</v>
+        <v>1.325</v>
       </c>
     </row>
     <row r="6">
@@ -1216,18 +1332,20 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026_07_10_14_05_42_11_case04_T6_P0.png</t>
+          <t>2026_07_09_12_13_04_11_case04_T6_P0.png</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>52.5335</v>
+        <v>51.416</v>
       </c>
       <c r="D6" t="n">
-        <v>1</v>
-      </c>
-      <c r="E6" t="inlineStr"/>
+        <v>16.7</v>
+      </c>
+      <c r="E6" t="n">
+        <v>1.292</v>
+      </c>
       <c r="F6" t="n">
-        <v>1</v>
+        <v>1.446</v>
       </c>
     </row>
   </sheetData>
@@ -1282,14 +1400,18 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026_07_10_13_07_04_11_case05_T8_P0.png</t>
+          <t>2026_07_09_10_17_50_11_case05_T8_P0.png</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>52.03</v>
-      </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
+        <v>51.0215</v>
+      </c>
+      <c r="D2" t="n">
+        <v>16.67</v>
+      </c>
+      <c r="E2" t="n">
+        <v>1.097</v>
+      </c>
       <c r="F2" t="n">
         <v>1.259</v>
       </c>
@@ -1300,18 +1422,20 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026_07_10_13_22_43_11_case05_T8_P0.png</t>
+          <t>2026_07_09_10_32_47_11_case05_T8_P0.png</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>51.983</v>
+        <v>51.092</v>
       </c>
       <c r="D3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E3" t="inlineStr"/>
+        <v>14.66</v>
+      </c>
+      <c r="E3" t="n">
+        <v>1.168</v>
+      </c>
       <c r="F3" t="n">
-        <v>1.291</v>
+        <v>1.334</v>
       </c>
     </row>
     <row r="4">
@@ -1320,18 +1444,20 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026_07_10_13_37_40_11_case05_T8_P0.png</t>
+          <t>2026_07_09_10_48_55_11_case05_T8_P0.png</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>51.9645</v>
+        <v>188.948</v>
       </c>
       <c r="D4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E4" t="inlineStr"/>
+        <v>16.06</v>
+      </c>
+      <c r="E4" t="n">
+        <v>1.142</v>
+      </c>
       <c r="F4" t="n">
-        <v>1.325</v>
+        <v>1.317</v>
       </c>
     </row>
     <row r="5">
@@ -1340,18 +1466,20 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026_07_10_13_52_07_11_case05_T8_P0.png</t>
+          <t>2026_07_09_11_43_59_11_case05_T8_P0.png</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>52.1185</v>
+        <v>51.405</v>
       </c>
       <c r="D5" t="n">
-        <v>1</v>
-      </c>
-      <c r="E5" t="inlineStr"/>
+        <v>16.55</v>
+      </c>
+      <c r="E5" t="n">
+        <v>1.151</v>
+      </c>
       <c r="F5" t="n">
-        <v>1.346</v>
+        <v>1.321</v>
       </c>
     </row>
     <row r="6">
@@ -1360,18 +1488,20 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026_07_10_14_07_08_11_case05_T8_P0.png</t>
+          <t>2026_07_09_12_14_29_11_case05_T8_P0.png</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>52.529</v>
+        <v>51.207</v>
       </c>
       <c r="D6" t="n">
-        <v>16.52</v>
-      </c>
-      <c r="E6" t="inlineStr"/>
+        <v>16.79</v>
+      </c>
+      <c r="E6" t="n">
+        <v>1.303</v>
+      </c>
       <c r="F6" t="n">
-        <v>1.343</v>
+        <v>1.458</v>
       </c>
     </row>
   </sheetData>
@@ -1426,18 +1556,20 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026_07_10_13_08_15_11_case06_T10_P0.png</t>
+          <t>2026_07_09_10_19_01_11_case06_T10_P0.png</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>40.5425</v>
+        <v>40.432</v>
       </c>
       <c r="D2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E2" t="inlineStr"/>
+        <v>16.68</v>
+      </c>
+      <c r="E2" t="n">
+        <v>1.12</v>
+      </c>
       <c r="F2" t="n">
-        <v>1.352</v>
+        <v>1.288</v>
       </c>
     </row>
     <row r="3">
@@ -1446,18 +1578,20 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026_07_10_13_23_53_11_case06_T10_P0.png</t>
+          <t>2026_07_09_10_33_58_11_case06_T10_P0.png</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>40.506</v>
+        <v>40.623</v>
       </c>
       <c r="D3" t="n">
-        <v>14.07</v>
-      </c>
-      <c r="E3" t="inlineStr"/>
+        <v>14.66</v>
+      </c>
+      <c r="E3" t="n">
+        <v>1.186</v>
+      </c>
       <c r="F3" t="n">
-        <v>1.373</v>
+        <v>1.362</v>
       </c>
     </row>
     <row r="4">
@@ -1466,16 +1600,20 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026_07_10_13_38_51_11_case06_T10_P0.png</t>
+          <t>2026_07_09_10_50_06_11_case06_T10_P0.png</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>2</v>
-      </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
+        <v>40.87</v>
+      </c>
+      <c r="D4" t="n">
+        <v>16.09</v>
+      </c>
+      <c r="E4" t="n">
+        <v>1.158</v>
+      </c>
       <c r="F4" t="n">
-        <v>1.422</v>
+        <v>1.339</v>
       </c>
     </row>
     <row r="5">
@@ -1484,16 +1622,20 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026_07_10_13_53_17_11_case06_T10_P0.png</t>
+          <t>2026_07_09_11_45_09_11_case06_T10_P0.png</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>40.6085</v>
-      </c>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
+        <v>40.723</v>
+      </c>
+      <c r="D5" t="n">
+        <v>16.62</v>
+      </c>
+      <c r="E5" t="n">
+        <v>1.157</v>
+      </c>
       <c r="F5" t="n">
-        <v>1.479</v>
+        <v>1.337</v>
       </c>
     </row>
     <row r="6">
@@ -1502,16 +1644,20 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026_07_10_14_08_19_11_case06_T10_P0.png</t>
+          <t>2026_07_09_12_15_40_11_case06_T10_P0.png</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>40.913</v>
-      </c>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
+        <v>40.72</v>
+      </c>
+      <c r="D6" t="n">
+        <v>16.74</v>
+      </c>
+      <c r="E6" t="n">
+        <v>1.324</v>
+      </c>
       <c r="F6" t="n">
-        <v>1.421</v>
+        <v>1.482</v>
       </c>
     </row>
   </sheetData>
@@ -1566,16 +1712,20 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026_07_10_13_09_13_11_case08_T18_P0.png</t>
+          <t>2026_07_09_10_54_48_11_case08_T18_P0.png</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>32.073</v>
-      </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
+        <v>89.866</v>
+      </c>
+      <c r="D2" t="n">
+        <v>38.14</v>
+      </c>
+      <c r="E2" t="n">
+        <v>1.207</v>
+      </c>
       <c r="F2" t="n">
-        <v>1.587</v>
+        <v>1.447</v>
       </c>
     </row>
     <row r="3">
@@ -1584,18 +1734,20 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026_07_10_13_24_52_11_case08_T18_P0.png</t>
+          <t>2026_07_09_11_15_09_11_case08_T18_P0.png</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>32.033</v>
+        <v>90.026</v>
       </c>
       <c r="D3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E3" t="inlineStr"/>
+        <v>37.4</v>
+      </c>
+      <c r="E3" t="n">
+        <v>1.235</v>
+      </c>
       <c r="F3" t="n">
-        <v>1.602</v>
+        <v>1.475</v>
       </c>
     </row>
     <row r="4">
@@ -1604,18 +1756,20 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026_07_10_13_39_49_11_case08_T18_P0.png</t>
+          <t>2026_07_09_11_30_54_11_case08_T18_P0.png</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>32.038</v>
+        <v>89.986</v>
       </c>
       <c r="D4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E4" t="inlineStr"/>
+        <v>36.74</v>
+      </c>
+      <c r="E4" t="n">
+        <v>1.234</v>
+      </c>
       <c r="F4" t="n">
-        <v>1.659</v>
+        <v>1.471</v>
       </c>
     </row>
     <row r="5">
@@ -1624,18 +1778,20 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026_07_10_13_54_16_11_case08_T18_P0.png</t>
+          <t>2026_07_09_11_46_09_11_case08_T18_P0.png</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>32.123</v>
+        <v>89.746</v>
       </c>
       <c r="D5" t="n">
-        <v>1</v>
-      </c>
-      <c r="E5" t="inlineStr"/>
+        <v>38.3</v>
+      </c>
+      <c r="E5" t="n">
+        <v>1.245</v>
+      </c>
       <c r="F5" t="n">
-        <v>1.689</v>
+        <v>1.474</v>
       </c>
     </row>
     <row r="6">
@@ -1644,18 +1800,20 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026_07_10_14_09_17_11_case08_T18_P0.png</t>
+          <t>2026_07_09_12_16_39_11_case08_T18_P0.png</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>32.3565</v>
+        <v>32.749</v>
       </c>
       <c r="D6" t="n">
-        <v>1</v>
-      </c>
-      <c r="E6" t="inlineStr"/>
+        <v>36.14</v>
+      </c>
+      <c r="E6" t="n">
+        <v>1.382</v>
+      </c>
       <c r="F6" t="n">
-        <v>1.647</v>
+        <v>1.596</v>
       </c>
     </row>
   </sheetData>
@@ -1710,16 +1868,20 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026_07_10_13_10_02_11_case09_T22_P1.png</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr"/>
+          <t>2026_07_09_10_19_45_11_case09_T22_P1.png</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>500</v>
+      </c>
       <c r="D2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E2" t="inlineStr"/>
+        <v>28.12</v>
+      </c>
+      <c r="E2" t="n">
+        <v>1.487</v>
+      </c>
       <c r="F2" t="n">
-        <v>1.726</v>
+        <v>1.802</v>
       </c>
     </row>
     <row r="3">
@@ -1728,18 +1890,20 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026_07_10_13_25_40_11_case09_T22_P1.png</t>
+          <t>2026_07_09_10_34_42_11_case09_T22_P1.png</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>45.9</v>
+        <v>20.324</v>
       </c>
       <c r="D3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E3" t="inlineStr"/>
+        <v>35.1</v>
+      </c>
+      <c r="E3" t="n">
+        <v>1.582</v>
+      </c>
       <c r="F3" t="n">
-        <v>1.779</v>
+        <v>1.91</v>
       </c>
     </row>
     <row r="4">
@@ -1748,16 +1912,20 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026_07_10_13_40_38_11_case09_T22_P1.png</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr"/>
+          <t>2026_07_09_10_50_50_11_case09_T22_P1.png</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>40.395</v>
+      </c>
       <c r="D4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E4" t="inlineStr"/>
+        <v>37.87</v>
+      </c>
+      <c r="E4" t="n">
+        <v>1.548</v>
+      </c>
       <c r="F4" t="n">
-        <v>1.841</v>
+        <v>1.886</v>
       </c>
     </row>
     <row r="5">
@@ -1766,18 +1934,20 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026_07_10_13_55_04_11_case09_T22_P1.png</t>
+          <t>2026_07_09_11_46_53_11_case09_T22_P1.png</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>21853</v>
+        <v>40.369</v>
       </c>
       <c r="D5" t="n">
-        <v>1</v>
-      </c>
-      <c r="E5" t="inlineStr"/>
+        <v>24.98</v>
+      </c>
+      <c r="E5" t="n">
+        <v>1.684</v>
+      </c>
       <c r="F5" t="n">
-        <v>1.848</v>
+        <v>1.995</v>
       </c>
     </row>
     <row r="6">
@@ -1786,16 +1956,20 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026_07_10_14_10_06_11_case09_T22_P1.png</t>
+          <t>2026_07_09_12_17_23_11_case09_T22_P1.png</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>22.009</v>
-      </c>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
+        <v>40.421</v>
+      </c>
+      <c r="D6" t="n">
+        <v>31.5175</v>
+      </c>
+      <c r="E6" t="n">
+        <v>1.733</v>
+      </c>
       <c r="F6" t="n">
-        <v>1.813</v>
+        <v>2.6</v>
       </c>
     </row>
   </sheetData>
@@ -1850,18 +2024,20 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026_07_10_13_10_50_11_case11_T28_P0.png</t>
+          <t>2026_07_09_10_20_33_11_case11_T28_P0.png</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>23.3095</v>
+        <v>21.792</v>
       </c>
       <c r="D2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E2" t="inlineStr"/>
+        <v>24.35</v>
+      </c>
+      <c r="E2" t="n">
+        <v>1.436</v>
+      </c>
       <c r="F2" t="n">
-        <v>1.844</v>
+        <v>1.732</v>
       </c>
     </row>
     <row r="3">
@@ -1870,16 +2046,20 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026_07_10_13_26_29_11_case11_T28_P0.png</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr"/>
+          <t>2026_07_09_10_35_31_11_case11_T28_P0.png</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>55.97</v>
+      </c>
       <c r="D3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E3" t="inlineStr"/>
+        <v>35.78</v>
+      </c>
+      <c r="E3" t="n">
+        <v>1.524</v>
+      </c>
       <c r="F3" t="n">
-        <v>1.886</v>
+        <v>1.831</v>
       </c>
     </row>
     <row r="4">
@@ -1888,18 +2068,20 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026_07_10_13_41_27_11_case11_T28_P0.png</t>
+          <t>2026_07_09_10_51_39_11_case11_T28_P0.png</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>23.287</v>
+        <v>21.965</v>
       </c>
       <c r="D4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E4" t="inlineStr"/>
+        <v>37.29</v>
+      </c>
+      <c r="E4" t="n">
+        <v>1.5605</v>
+      </c>
       <c r="F4" t="n">
-        <v>1.949</v>
+        <v>1.825</v>
       </c>
     </row>
     <row r="5">
@@ -1908,18 +2090,20 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026_07_10_13_55_53_11_case11_T28_P0.png</t>
+          <t>2026_07_09_11_47_42_11_case11_T28_P0.png</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>23.346</v>
+        <v>54.53</v>
       </c>
       <c r="D5" t="n">
-        <v>1</v>
-      </c>
-      <c r="E5" t="inlineStr"/>
+        <v>26.37</v>
+      </c>
+      <c r="E5" t="n">
+        <v>1.623</v>
+      </c>
       <c r="F5" t="n">
-        <v>1.968</v>
+        <v>1.914</v>
       </c>
     </row>
     <row r="6">
@@ -1928,14 +2112,20 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026_07_10_14_10_54_11_case11_T28_P0.png</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
+          <t>2026_07_09_12_18_12_11_case11_T28_P0.png</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>21.815</v>
+      </c>
+      <c r="D6" t="n">
+        <v>25.21</v>
+      </c>
+      <c r="E6" t="n">
+        <v>1.659</v>
+      </c>
       <c r="F6" t="n">
-        <v>1.909</v>
+        <v>1.944</v>
       </c>
     </row>
   </sheetData>

</xml_diff>